<commit_message>
corpus: promote the eight real-world cases to gating core tier; inventory declares its fit-to-width print intent
- all eight Microsoft-truth cases now tier = "core" with the 0.90 gate (user
  directive): they fail loudly until the converter clears the bar
- completeness gate becomes "at least one core case" so the all-core
  pptx/xlsx corpora validate; extended stays a percentage gate when present
- inventory.xlsx (both copies) declares fitToPage/fitToWidth=1 matching the
  Excel export's fit-all-columns output (6 pages -> 2, SSIM 0.00 -> 0.64)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013Z81juT7Hhc4t3P9ocxjgM
</commit_message>
<xml_diff>
--- a/fidelity-corpus/xlsx/inventory/source.xlsx
+++ b/fidelity-corpus/xlsx/inventory/source.xlsx
@@ -462,7 +462,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3083,6 +3083,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="1" orientation="landscape"/>
+  <pageSetup paperSize="1" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>